<commit_message>
Updated existing Data, Individual level logic later.
</commit_message>
<xml_diff>
--- a/docs/Logic Requirements/Ageipelago Joan of Arc.xlsx
+++ b/docs/Logic Requirements/Ageipelago Joan of Arc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/BB6DD295C338E39F/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefb\OneDrive\Desktop\Logic Requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{BA2542DF-DBA3-4D13-8D9D-81B85B6B4E30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38727B9F-1E22-4033-AAF8-5C72A93D96F7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B2EA931-9906-47E9-82BD-7BDE5EAB488E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9E5C4DF5-6A70-45B6-8795-4F3A15A3E9BB}"/>
   </bookViews>
@@ -37,33 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
-  <si>
-    <r>
-      <t xml:space="preserve">Once again, we might want to split Siege from non-Siege units for items.
-The additional Resources are given when destroying </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Burgundies Town Center</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, with the wood dependeing on their leftover Resources in Vanilla.</t>
-    </r>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
   <si>
     <t>6 Villagers</t>
   </si>
@@ -74,62 +48,10 @@
 100 Wood</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve"> Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundies northern Town Center</t>
-    </r>
-  </si>
-  <si>
     <t>Bring the Cart carrying the French Flag to the flagged Hill</t>
   </si>
   <si>
     <t>A Perfect Martyr</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">BIG Scenario.
-I suggest seperating the starting army's siege and regular units.
-Not sure if the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>King's Men</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> CAN be defeated, but it SHOULD be possible.
-Lots of Enemies here, so I figured we'd do well to split them up into multiple Objectives.</t>
-    </r>
-  </si>
-  <si>
-    <t>10 Men-at-Arms
-2 Throwing Axemen
-2 Knights
-2 Heavy Scorpions</t>
-  </si>
-  <si>
-    <t>6 Villagers
-4 Villagers</t>
   </si>
   <si>
     <t>Joan of Arc
@@ -148,154 +70,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Optain 10 Villagers
-Bring 10 Villagers to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF06CFEA"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Compiègne</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>1/2/3 English Castle/s</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat all </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>English Units south of the River</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat all </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>English units North of the River</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>English</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundy</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>King's Men</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF06CFEA"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Compiègne</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Optain at least 6 Villagers
 Meet </t>
     </r>
@@ -330,13 +104,6 @@
   </si>
   <si>
     <t>The Siege of Paris</t>
-  </si>
-  <si>
-    <t>Misc. Buildings</t>
-  </si>
-  <si>
-    <t>6 Villagers
-1 Town Center</t>
   </si>
   <si>
     <t>Joan of Arc
@@ -352,141 +119,10 @@
 150 Stone</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Rheims</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Chalons</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Troyes</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>English Guards</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>the Town Center of Rheims</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>the Town Center of Chalons</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>the Town Center of Troyes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Reach the French Town</t>
-    </r>
-  </si>
-  <si>
     <t>The Rising</t>
   </si>
   <si>
     <t>I recommend making the Villagers or Resources an item, as only these 2 are needed for Vicory.</t>
-  </si>
-  <si>
-    <t>2 Transport Ships, 2 Demolition Ships</t>
   </si>
   <si>
     <t>Joan of Arc
@@ -502,124 +138,6 @@
 150 Stone</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>4 English Castles</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>English</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Fastolf's Army</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundy</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>1/2 English Castle/s</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Kill </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Sir John Fastolf</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>3 English Castles</t>
-    </r>
-  </si>
-  <si>
     <t>The Cleansing of the Loire</t>
   </si>
   <si>
@@ -630,359 +148,12 @@
 1 Scout Cavalry</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>2/3/4 English</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Castle/s</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Northern Englis</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">h
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Southern English</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundy</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Chinon</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF06CFEA"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Blois</t>
-    </r>
-  </si>
-  <si>
     <t>The Maid of Orleans</t>
-  </si>
-  <si>
-    <t>Due to how powerfull they are, I would recommend turning the 2 hero knights in the starting units into an item, as they can kill just about everything on the map when used properly.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>4 Men-at-Arms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (first camp)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>4 Crossbowmen</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (first camp)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>4 Men-at-Arms, 6 Pikemen, 1 Capped Ram</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (second camp)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>6 Crossbowmen, 2 Scorpions</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (third camp)</t>
-    </r>
-  </si>
-  <si>
-    <t>2 Transport Ships</t>
   </si>
   <si>
     <t>Joan the Maid
 Sieur Bertrand
 Sieur de Metz</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Highwaymen</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Destroy the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundian Castle</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundian Ambush</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundy</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Army of France</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Chinon</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Enter the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Burgundian Village</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Bring Joan to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Chinon</t>
-    </r>
   </si>
   <si>
     <t>An unlikely Messiah</t>
@@ -1741,232 +912,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> and destroy their Castles.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>6 Trade Carts (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF06CFEA"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Blois</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>)
-3 Villagers (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Orlèans</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>)
-1 Town Center (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Orlèans</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>12 Crossbowmen, 8 Knights (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF03CBF3"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Blois</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>)
-2 Transport Ships, 1 Dock
-Misc. Buildings (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Orlèans</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>)
-1000 Food, 1500 Wood, 1500 Gold, 500 Stone</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Defeating </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Orléans</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> would be pointless, seeing as they only own the Cathedral that must survive.
-The Resources are given when the Trade Carts reach </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Orlèans</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Bring Joan to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF06CFEA"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Blois</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Bring 6 Trade Carts to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Orlèans</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Bring Joan to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="0" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Orléans</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Destroy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">1 English </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Castle</t>
     </r>
   </si>
   <si>
@@ -3103,11 +2048,6 @@
     </r>
   </si>
   <si>
-    <t>La Hire, Constable Richemont, 16 Arbalesters, 8 Champions, 8 Hussars, 6 Paladins, 2 Trebuchets (1 on Hard) (French Army)
-Jean Bureau, 8 Hand Cannoneers, 6 Bombard Cannons (3 on Hard) (French Artillery)
-400 Food, 400 Wood, 50 Gold, 150 Stone</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Reach the French Army
 Reach the French Artillery
@@ -3333,6 +2273,1248 @@
       </rPr>
       <t xml:space="preserve"> and reaching the Hill with the Flag is possible when the Player can build a base.</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4 Men-at-Arms,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4 Crossbowmen</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (first camp)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4 Men-at-Arms, 6 Pikemen, 1 Capped Ram</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (second camp)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>6 Crossbowmen, 2 Scorpions</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (third camp)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Castles</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Reach the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Western Units</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Reach the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Southern Units</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Reach the Transport Ships
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Burgundy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Army of France</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Chinon
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Defeat</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Highwaymen</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bring Joan the Maid to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Chinon</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2/3/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF03CBF3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>English Castle/s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Northern English</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Southern English</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Burgundy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Chinon</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF06CFEA"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Blois</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Castles</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1/2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Castle/s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Kill </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Sir John Fastolf</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Castles</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>English</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Fastolf's Army</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Burgundy</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Rheims'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Chalons'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Troyes' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Town Center</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Reach the French Town</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Rheims</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Chalons</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Troyes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> English Guards</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bring Joan of Arc to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Orléans</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>English Castle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Bring Joan of Arc to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF03CBF3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Blois</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Bring 6 Trade Carts to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Orlèans</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>12 Crossbowmen, 8 Knights (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF03CBF3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Blois</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>)
+2 Transport Ships, 1 Dock (Gaia)
+1000 Food, 1500 Wood, 1500 Gold, 500 Stone</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>6 Trade Carts (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF06CFEA"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Blois</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>)
+3 Villagers, 1 Town Center, Misc. Buildings (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Orlèans</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Defeating </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Orléans</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> would be pointless, seeing as they only own the Cathedral that must survive.
+In Vanilla the Resources are given when the Trade Carts reach </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Orlèans</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Burgundys </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>northern Town Center</t>
+    </r>
+  </si>
+  <si>
+    <t>6 Villagers
+4 Villagers
+(Gaia)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+Bring 10 Villagers to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF06CFEA"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Compiègne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Destroy </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1/2/3/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF03CBF3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Castle/s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Kill all </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">English </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Units</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>south of the River</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Kill all </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">English </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Units</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>North of the River</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>English</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Burgundy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>King's Men</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF06CFEA"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Compiègne</t>
+    </r>
+  </si>
+  <si>
+    <t>2 Transport Ships
+(Gaia)</t>
+  </si>
+  <si>
+    <t>2 Transport Ships, 2 Demolition Ships (Gaia)</t>
+  </si>
+  <si>
+    <t>6 Villagers, 1 Town Center, Misc. Buildings
+(Gaia)</t>
+  </si>
+  <si>
+    <r>
+      <t>10 Men-at-Arms, 2 Throwing Axemen, 2 Knights, 2 Heavy Scorpions
+(Gaia)
+1 Militia, 1 Scout (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>King's Men</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>La Hire, Constable Richemont, 16 Arbalesters, 8 Champions, 8 Hussars, 6 Paladins, 2 Trebuchets (1 on Hard)
+Jean Bureau, 8 Hand Cannoneers, 6 Bombard Cannons (3 on Hard)
+(Gaia)
+400 Food, 400 Wood, 50 Gold, 150 Stone
+Walls, Gates (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Burgundy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Once again, we might want to split Siege from non-Siege Units for Items.
+The additional Resources are given when destroying </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Burgundies Town Center</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, with the Wood dependeing on their leftover Resources in Vanilla.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BIG Scenario.
+I suggest seperating the Starting Army's Siege and regular Units.
+Not sure if the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>King's Men</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> CAN be defeated, but it SHOULD be possible.
+Lots of Enemies here, so I figured we'd do well to split them up into multiple Objectives.</t>
+    </r>
+  </si>
+  <si>
+    <t>Due to how powerfull they are, I would recommend turning the 2 Hero Knights in the starting Units into an Item, as they can kill just about everything on the Map when used properly.</t>
   </si>
 </sst>
 </file>
@@ -3418,19 +3600,6 @@
     </font>
     <font>
       <sz val="18"/>
-      <color rgb="FF3A3A3A"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color rgb="FF3A3A3A"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -3501,6 +3670,17 @@
       <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -3603,7 +3783,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3617,12 +3797,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3632,13 +3806,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3983,307 +4166,299 @@
   <sheetData>
     <row r="2" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:17" ht="70.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="12" t="s">
-        <v>45</v>
+      <c r="B3" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="L3" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="M3" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="O3" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="P3" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q3" s="10" t="s">
-        <v>53</v>
+        <v>18</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="6" t="s">
+    <row r="4" spans="2:17" ht="375.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5" t="s">
         <v>37</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="5" spans="2:17" ht="375.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="6" t="s">
-        <v>29</v>
+      <c r="B5" s="11" t="s">
+        <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>68</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7" t="s">
-        <v>64</v>
+        <v>73</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:17" ht="338.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="5" t="s">
-        <v>26</v>
+      <c r="B6" s="12" t="s">
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2" t="s">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7" t="s">
-        <v>73</v>
+        <v>9</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="2:17" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="4" t="s">
-        <v>19</v>
+      <c r="B7" s="11" t="s">
+        <v>8</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="H7" s="2"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="7" t="s">
-        <v>77</v>
+      <c r="J7" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="2:17" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="4" t="s">
-        <v>12</v>
+      <c r="B8" s="11" t="s">
+        <v>6</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>10</v>
+        <v>76</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="2:17" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>4</v>
+      <c r="B9" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>3</v>
+        <v>74</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7" t="s">
-        <v>88</v>
+        <v>82</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>